<commit_message>
Add evaluation notebook for SE-ResNeXt-50 YOLO ROI test and update experiment summary
- Created a new Jupyter notebook for evaluating the SE-ResNeXt-50 model on the locked YOLO ROI test split, including metrics, confusion matrix, and Grad-CAM visualizations.
- Added a detailed evaluation configuration and preprocessing steps to ensure reproducibility.
- Implemented a new dataset class for loading test images and their corresponding labels.
- Loaded the model checkpoint and performed inference, saving predictions and metrics to CSV and JSON files.
- Enhanced the experiment summary script with a new entry for DenseNet-121 validation production-ROI robustness fine-tune, detailing model parameters and evaluation metrics.
- Updated the KL response viewer to change the label from "Native CAM heatmap" to "Class activation heatmap" for clarity.
</commit_message>
<xml_diff>
--- a/docs/report/all_experiments.xlsx
+++ b/docs/report/all_experiments.xlsx
@@ -44,7 +44,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-28T04:43:20.483245+00:00</t>
+          <t>2026-07-31T08:56:55.608703+00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -61,7 +61,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>all_runs=36; DenseNet=26; SE-ResNeXt=6; EfficientNet=1; deployment=3</t>
+          <t>all_runs=34; DenseNet=24; SE-ResNeXt=6; EfficientNet=1; deployment=3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_121/assets/2026-07-25_15-32-33_UTC_api_cam_localization_audit/report.md</t>
+          <t>docs/report/dense_net_121/2026-07-29_dataset_paper_lineage_summary.md</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_121/joint_guided_cam_run_2026-07-22.md</t>
+          <t>docs/report/dense_net_121/2026-07-29_densenet121_metric_gradcam_design_review.md</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_121/localization_strategy_proposal.md</t>
+          <t>docs/report/dense_net_121/2026-07-30_glcm_experiment_plan.md</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_121/native_cam_method_and_references.md</t>
+          <t>docs/report/dense_net_121/assets/2026-07-25_15-32-33_UTC_api_cam_localization_audit/report.md</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_121/report.md</t>
+          <t>docs/report/dense_net_121/joint_guided_cam_run_2026-07-22.md</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_201/dense_net_201_configuration_guide.md</t>
+          <t>docs/report/dense_net_121/localization_strategy_proposal.md</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
+          <t>docs/report/dense_net_121/native_cam_method_and_references.md</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>docs/report/efficientnet_b0/report.md</t>
+          <t>docs/report/dense_net_121/report.md</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -835,7 +835,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>docs/report/ensemble/2026-07-24_09-03-08_three_model_weighted_soft_voting.md</t>
+          <t>docs/report/efficientnet_b0/report.md</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>docs/report/ensemble/2026-07-24_16-50-26_365170_UTC_deployed_api_full_test.md</t>
+          <t>docs/report/se_resnext50_32x4d/report.md</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -879,110 +879,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>docs/report/se_resnext50_32x4d/report.md</t>
+          <t>notebooks/experiments/densenet121/heatmaps/dense_net_121_roi_robustness_ablation.ipynb</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>report markdown</t>
+          <t>notebook</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>source report</t>
+          <t>planned/not run</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
           <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>notebooks/experiments/dense_net_121_roi_robustness_ablation.ipynb</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>notebook</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>planned/not run</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>md</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>completed run artifact</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/arm_comparison.csv</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>csv</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>completed run artifact</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/gradcam_comparison_summary.json</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>completed run artifact</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495 UTC</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5277,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5375,17 +5287,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Test whether small YOLO ROI expansion and centre-shift variation reduces border-dependent Grad-CAM.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Do not replace the paired-view production checkpoint: metrics improved but aggregate CAM border energy increased.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5395,22 +5307,22 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
+          <t>inverse-frequency WeightedRandomSampler</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
+          <t>five-epoch full fine-tune</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
+          <t>Horizontal flip p=0.50; rotation +/-5; brightness/contrast 0.08; RandomErasing p=0.10</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
+          <t>Grad-CAM at DenseNet features.norm5</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -5439,148 +5351,146 @@
         </is>
       </c>
       <c r="Q34">
-        <v>0.8126277960220584</v>
+        <v>0.7650</v>
       </c>
       <c r="R34">
-        <v>0.6819234872143023</v>
-      </c>
-      <c r="S34">
-        <v>0.45751633986928103</v>
+        <v>0.6451</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="T34">
-        <v>0.7430301895958674</v>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X34">
-        <v>0.020581113801452784</v>
+        <v>0.6756</v>
+      </c>
+      <c r="U34">
+        <v>0.8505</v>
+      </c>
+      <c r="V34">
+        <v>0.0844</v>
+      </c>
+      <c r="W34">
+        <v>1.0000</v>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth</t>
+          <t/>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>aa774a2fc765244e03d29e622e31ce0f8fa33a27aeaae8fbf5c5ec312f447fc2</t>
+          <t/>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>completed; not promoted</t>
+          <t>completed; separate model report</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Cross-Entropy (CE)</t>
+          <t>CORN; Focal CORN in final stage</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
+          <t>Balanced WeightedRandomSampler in warm-up/coarse stages; stage-3 natural skew</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
+          <t>3-stage warm-up + coarse + fine-tune</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
+          <t>Horizontal flip p=0.50; capped rotation; small RandomErasing; no color jitter</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>Grad-CAM over norm5</t>
+        </is>
+      </c>
+      <c r="L35">
+        <v>0.6624</v>
+      </c>
+      <c r="M35">
+        <v>0.7763</v>
+      </c>
+      <c r="N35">
+        <v>0.63</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q35">
-        <v>0.8202226229712083</v>
-      </c>
-      <c r="R35">
-        <v>0.68151148175952</v>
-      </c>
-      <c r="S35">
-        <v>0.43137254901960786</v>
-      </c>
-      <c r="T35">
-        <v>0.7438495789896049</v>
+      <c r="P35">
+        <v>0.6948</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
@@ -5597,291 +5507,27 @@
           <t/>
         </is>
       </c>
-      <c r="X35">
-        <v>0.01937046004842615</v>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>288 / 826</t>
+        </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth</t>
+          <t>checkpoints/densenet201/best_model.pth</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>f955d0f516cd30d3c057c822e97219841e24da74dabbbc9f5dad134a31b43dd6</t>
+          <t>a8107b9cc7cc9242385f1facfcfc69c251f88697ed2df4dae8a43c1d66729b76</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
-        <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>DenseNet-121</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>completed; not promoted</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Cross-Entropy (CE)</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q36">
-        <v>0.8037057762855189</v>
-      </c>
-      <c r="R36">
-        <v>0.6832540391938888</v>
-      </c>
-      <c r="S36">
-        <v>0.49019607843137253</v>
-      </c>
-      <c r="T36">
-        <v>0.7298324958134197</v>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X36">
-        <v>0.026634382566585957</v>
-      </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>0c26982e344a339c247d4fc7d3a65672cade9c912d9f7f51b7f1a3256c430b28</t>
-        </is>
-      </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-      <c r="AB36" t="inlineStr">
-        <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>completed; separate model report</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>CORN; Focal CORN in final stage</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Balanced WeightedRandomSampler in warm-up/coarse stages; stage-3 natural skew</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>3-stage warm-up + coarse + fine-tune</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Horizontal flip p=0.50; capped rotation; small RandomErasing; no color jitter</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Grad-CAM over norm5</t>
-        </is>
-      </c>
-      <c r="L37">
-        <v>0.6624</v>
-      </c>
-      <c r="M37">
-        <v>0.7763</v>
-      </c>
-      <c r="N37">
-        <v>0.63</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P37">
-        <v>0.6948</v>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>288 / 826</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>checkpoints/densenet201/best_model.pth</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>a8107b9cc7cc9242385f1facfcfc69c251f88697ed2df4dae8a43c1d66729b76</t>
-        </is>
-      </c>
-      <c r="AA37" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-      <c r="AB37" t="inlineStr">
         <is>
           <t>DenseNet-201 report recommends balanced stage-3 training and threshold review, but those recommendations were not validated in the documented run.</t>
         </is>
@@ -9087,7 +8733,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -9097,7 +8743,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>validation/CAM ablation</t>
+          <t>validation production-ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -9107,42 +8753,42 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Test whether small YOLO ROI expansion and centre-shift variation reduces border-dependent Grad-CAM.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Do not replace the paired-view production checkpoint: metrics improved but aggregate CAM border energy increased.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
+          <t>docs/AI_REPORT.md</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth</t>
+          <t>Google Drive: Models/densenet121_production_roi_robustness/2026-07-30_15-45-03_830205_UTC</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth</t>
+          <t/>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>aa774a2fc765244e03d29e622e31ce0f8fa33a27aeaae8fbf5c5ec312f447fc2</t>
+          <t/>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>timm_densenet121_linear_native_cam</t>
+          <t>timm_densenet121_linear_gradcam</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -9167,79 +8813,79 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>manual_artifact_metadata</t>
+          <t>executed_notebook</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>UTC</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>validation/CAM ablation</t>
+          <t>training/evaluation report</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>completed; not promoted</t>
+          <t>completed; separate model report</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth</t>
+          <t>checkpoints/densenet201</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth</t>
+          <t>checkpoints/densenet201/best_model.pth</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>f955d0f516cd30d3c057c822e97219841e24da74dabbbc9f5dad134a31b43dd6</t>
+          <t>a8107b9cc7cc9242385f1facfcfc69c251f88697ed2df4dae8a43c1d66729b76</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>timm_densenet121_linear_native_cam</t>
+          <t>Multi-scale DenseNet-201; pooled transition-2, transition-3, and norm5 features</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -9264,204 +8910,10 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
-        <is>
-          <t>manual_artifact_metadata</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>DenseNet-121</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>UTC</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>validation/CAM ablation</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>completed; not promoted</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>0c26982e344a339c247d4fc7d3a65672cade9c912d9f7f51b7f1a3256c430b28</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>timm_densenet121_linear_native_cam</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>manual_artifact_metadata</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>training/evaluation report</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>completed; separate model report</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>checkpoints/densenet201</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>checkpoints/densenet201/best_model.pth</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>a8107b9cc7cc9242385f1facfcfc69c251f88697ed2df4dae8a43c1d66729b76</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>Multi-scale DenseNet-201; pooled transition-2, transition-3, and norm5 features</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
         <is>
           <t>report_markdown</t>
         </is>
@@ -18384,7 +17836,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -18394,7 +17846,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>validation/CAM ablation</t>
+          <t>validation production-ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -18404,106 +17856,106 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Test whether small YOLO ROI expansion and centre-shift variation reduces border-dependent Grad-CAM.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Do not replace the paired-view production checkpoint: metrics improved but aggregate CAM border energy increased.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>No labeled test evaluation in this run; external YOLO-crop shift remains unresolved.</t>
+          <t>CAM energy masks are broad geometry heuristics, not expert lesion annotations.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
+          <t>docs/AI_REPORT.md</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>not archived in report folder</t>
+          <t>notebooks/experiments/densenet121/roi/dense_net_121_production_roi_robustness.ipynb</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth</t>
+          <t>Google Drive: Models/densenet121_production_roi_robustness/2026-07-30_15-45-03_830205_UTC</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>timm_densenet121_linear_native_cam</t>
+          <t>timm_densenet121_linear_gradcam</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>ImageNet pretrained</t>
+          <t>paired-view DenseNet-121 CE checkpoint</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>384x384 direct resize after square pad</t>
+          <t>384x384</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Complete square-padded knee ROI; no center crop</t>
+          <t>YOLO box; train random expansion 1.10-1.20 and shift up to 5%; validation fixed 1.15 square; external black padding only</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>LAB CLAHE clipLimit 1.25; SquarePad; direct Resize 384; ImageNet normalization</t>
+          <t>LAB CLAHE 1.25; SquarePad; Resize 384; ImageNet normalization</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
+          <t>Horizontal flip p=0.50; rotation +/-5; brightness/contrast 0.08; RandomErasing p=0.10</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Deterministic square-pad/CLAHE/resize; no stochastic augmentation</t>
+          <t>Fixed production ROI and deterministic preprocessing; test set not opened</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Natural left/right orientation; no deterministic mirroring</t>
+          <t>Natural orientation; no deterministic mirroring</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
+          <t>inverse-frequency WeightedRandomSampler</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
+          <t>five-epoch full fine-tune</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>5 head warm-up; 15 coarse; 10 full fine-tune</t>
+          <t>full model fine-tune</t>
         </is>
       </c>
       <c r="X24">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Y24">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="Z24">
         <v>48</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>4 / Tesla T4</t>
+          <t>2 / CUDA</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -18528,12 +17980,12 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>warm-up 3e-4; coarse backbone 3e-5/head 3e-4; fine-tune 1e-5</t>
+          <t>1e-5</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>1e-4</t>
+          <t>1e-3</t>
         </is>
       </c>
       <c r="AH24" t="inlineStr">
@@ -18548,7 +18000,7 @@
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t/>
         </is>
       </c>
       <c r="AK24">
@@ -18561,17 +18013,17 @@
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
+          <t>Grad-CAM at DenseNet features.norm5</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>12x12</t>
+          <t>12x12 upsampled to 384x384</t>
         </is>
       </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>5,778 train / 826 validation; test not read</t>
+          <t>5,778 train / 826 validation; 227 deterministic CAM audit cases; test not opened</t>
         </is>
       </c>
       <c r="AP24" t="inlineStr">
@@ -18644,22 +18096,22 @@
           <t/>
         </is>
       </c>
-      <c r="BD24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="BD24">
+        <v>0.6186</v>
       </c>
       <c r="BE24">
-        <v>0.8126277960220584</v>
+        <v>0.7650</v>
       </c>
       <c r="BF24">
-        <v>0.6819234872143023</v>
-      </c>
-      <c r="BG24">
-        <v>0.45751633986928103</v>
+        <v>0.6451</v>
+      </c>
+      <c r="BG24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="BH24">
-        <v>0.7430301895958674</v>
+        <v>0.6756</v>
       </c>
       <c r="BI24" t="inlineStr">
         <is>
@@ -18667,33 +18119,27 @@
         </is>
       </c>
       <c r="BJ24">
-        <v>0.762976862415803</v>
+        <v>0.7156</v>
       </c>
       <c r="BK24">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="BL24">
-        <v>826</v>
-      </c>
-      <c r="BM24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>227</v>
+      </c>
+      <c r="BM24">
+        <v>0.8505</v>
+      </c>
+      <c r="BN24">
+        <v>0.0844</v>
       </c>
       <c r="BO24" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="BP24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="BP24">
+        <v>1.0000</v>
       </c>
       <c r="BQ24" t="inlineStr">
         <is>
@@ -18707,11 +18153,13 @@
       </c>
       <c r="BS24" t="inlineStr">
         <is>
-          <t>Anatomy-gate failure rate 2.0581%; see per-case CSV in run folder.</t>
-        </is>
-      </c>
-      <c r="BT24">
-        <v>0.020581113801452784</v>
+          <t>Baseline: joint energy 0.8648, border energy 0.0761, peak-inside 0.9956. Candidate did not meet CAM promotion rule.</t>
+        </is>
+      </c>
+      <c r="BT24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="BU24" t="inlineStr">
         <is>
@@ -18730,102 +18178,104 @@
       </c>
       <c r="BX24" t="inlineStr">
         <is>
-          <t>{"arm": "aggressive_double_cutout", "best_epoch": "27", "cam_failure_rate": "0.020581113801452784", "checkpoint": "/content/drive/MyDrive/Models/densenet121_checkpoints/2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth", "grade1_recall": "0.45751633986928103", "macro_ap": "0.7430301895958674", "macro_f1": "0.6819234872143023", "qwk": "0.8126277960220584", "selection_score": "0.762976862415803"}</t>
+          <t/>
         </is>
       </c>
       <c r="BY24" t="inlineStr">
         <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
+          <t/>
         </is>
       </c>
       <c r="BZ24" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
       <c r="CA24" t="inlineStr">
         <is>
-          <t>manual_artifact_metadata</t>
+          <t>executed_notebook</t>
         </is>
       </c>
       <c r="CB24" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_double_cutout/best_model.pth</t>
+          <t/>
         </is>
       </c>
       <c r="CC24" t="inlineStr">
         <is>
-          <t>aa774a2fc765244e03d29e622e31ce0f8fa33a27aeaae8fbf5c5ec312f447fc2</t>
-        </is>
-      </c>
-      <c r="CD24">
-        <v>27</v>
+          <t/>
+        </is>
+      </c>
+      <c r="CD24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>UTC</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>validation/CAM ablation</t>
+          <t>training/evaluation report</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>completed; not promoted</t>
+          <t>completed; separate model report</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
+          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
+          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>No labeled test evaluation in this run; external YOLO-crop shift remains unresolved.</t>
+          <t>Report does not provide an exact UTC run timestamp or checkpoint provenance; do not use as an exact production record.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>not archived in report folder</t>
+          <t>dense_net_201.ipynb (path not present in report folder)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth</t>
+          <t>checkpoints/densenet201</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>timm_densenet121_linear_native_cam</t>
+          <t>Multi-scale DenseNet-201; pooled transition-2, transition-3, and norm5 features</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -18835,66 +18285,70 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>384x384 direct resize after square pad</t>
+          <t>300x300</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Complete square-padded knee ROI; no center crop</t>
+          <t>Square-padded knee ROI; exact crop provenance not documented</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>LAB CLAHE clipLimit 1.25; SquarePad; direct Resize 384; ImageNet normalization</t>
+          <t>Square padding; CLAHE; grayscale normalization; resize as configured</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
+          <t>Horizontal flip p=0.50; capped rotation; small RandomErasing; no color jitter</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Deterministic square-pad/CLAHE/resize; no stochastic augmentation</t>
+          <t>Deterministic preprocessing; exact sequence not fully recorded</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Natural left/right orientation; no deterministic mirroring</t>
+          <t>Natural/symmetric laterality; exact policy not recorded</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
+          <t>Balanced WeightedRandomSampler in warm-up/coarse stages; stage-3 natural skew</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
+          <t>3-stage warm-up + coarse + fine-tune</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>5 head warm-up; 15 coarse; 10 full fine-tune</t>
+          <t>5 head warm-up; 25 coarse; 15 focal-CORN fine-tune (per configuration guide)</t>
         </is>
       </c>
       <c r="X25">
-        <v>30</v>
-      </c>
-      <c r="Y25">
-        <v>29</v>
-      </c>
-      <c r="Z25">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>4 / Tesla T4</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Cross-Entropy (CE)</t>
+          <t>CORN; Focal CORN in final stage</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -18909,71 +18363,67 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>CosineAnnealingLR</t>
+          <t>Cosine annealing; eta_min 1e-7</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>warm-up 3e-4; coarse backbone 3e-5/head 3e-4; fine-tune 1e-5</t>
+          <t>backbone 1e-5; head 1e-4; final 1e-5</t>
         </is>
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>1e-4</t>
+          <t>1e-4 stages 1/2; 1e-3 stage 3</t>
         </is>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>CUDA AMP</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>global norm 1.0</t>
+          <t/>
         </is>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="AK25">
-        <v>42</v>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
       </c>
       <c r="AL25" t="inlineStr">
         <is>
-          <t>0.55 QWK + 0.30 macro F1 + 0.15 macro AP</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="AM25" t="inlineStr">
         <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
+          <t>Grad-CAM over norm5</t>
         </is>
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>12x12</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="AO25" t="inlineStr">
         <is>
-          <t>5,778 train / 826 validation; test not read</t>
-        </is>
-      </c>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AQ25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>1,656-image test split; patient grouping not documented</t>
+        </is>
+      </c>
+      <c r="AP25">
+        <v>1656</v>
+      </c>
+      <c r="AQ25">
+        <v>0.6624</v>
+      </c>
+      <c r="AR25">
+        <v>0.7763</v>
       </c>
       <c r="AS25" t="inlineStr">
         <is>
@@ -18990,10 +18440,8 @@
           <t/>
         </is>
       </c>
-      <c r="AV25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AV25">
+        <v>0.63</v>
       </c>
       <c r="AW25" t="inlineStr">
         <is>
@@ -19005,15 +18453,11 @@
           <t/>
         </is>
       </c>
-      <c r="AY25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AZ25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AY25">
+        <v>0.6948</v>
+      </c>
+      <c r="AZ25">
+        <v>0.8812</v>
       </c>
       <c r="BA25" t="inlineStr">
         <is>
@@ -19035,31 +18479,45 @@
           <t/>
         </is>
       </c>
-      <c r="BE25">
-        <v>0.8202226229712083</v>
-      </c>
-      <c r="BF25">
-        <v>0.68151148175952</v>
-      </c>
-      <c r="BG25">
-        <v>0.43137254901960786</v>
-      </c>
-      <c r="BH25">
-        <v>0.7438495789896049</v>
+      <c r="BE25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BF25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BG25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BH25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="BI25" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="BJ25">
-        <v>0.7671533240104613</v>
-      </c>
-      <c r="BK25">
-        <v>29</v>
-      </c>
-      <c r="BL25">
-        <v>826</v>
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="BM25" t="inlineStr">
         <is>
@@ -19093,11 +18551,13 @@
       </c>
       <c r="BS25" t="inlineStr">
         <is>
-          <t>Anatomy-gate failure rate 1.9370%; see per-case CSV in run folder.</t>
-        </is>
-      </c>
-      <c r="BT25">
-        <v>0.01937046004842615</v>
+          <t/>
+        </is>
+      </c>
+      <c r="BT25" t="inlineStr">
+        <is>
+          <t>288 / 826</t>
+        </is>
       </c>
       <c r="BU25" t="inlineStr">
         <is>
@@ -19116,817 +18576,35 @@
       </c>
       <c r="BX25" t="inlineStr">
         <is>
-          <t>{"arm": "aggressive_single_cutout", "best_epoch": "29", "cam_failure_rate": "0.01937046004842615", "checkpoint": "/content/drive/MyDrive/Models/densenet121_checkpoints/2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth", "grade1_recall": "0.43137254901960786", "macro_ap": "0.7438495789896049", "macro_f1": "0.68151148175952", "qwk": "0.8202226229712083", "selection_score": "0.7671533240104613"}</t>
+          <t/>
         </is>
       </c>
       <c r="BY25" t="inlineStr">
         <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
+          <t>DenseNet-201 report recommends balanced stage-3 training and threshold review, but those recommendations were not validated in the documented run.</t>
         </is>
       </c>
       <c r="BZ25" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
       <c r="CA25" t="inlineStr">
         <is>
-          <t>manual_artifact_metadata</t>
+          <t>report_markdown</t>
         </is>
       </c>
       <c r="CB25" t="inlineStr">
         <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/aggressive_single_cutout/best_model.pth</t>
+          <t>checkpoints/densenet201/best_model.pth</t>
         </is>
       </c>
       <c r="CC25" t="inlineStr">
         <is>
-          <t>f955d0f516cd30d3c057c822e97219841e24da74dabbbc9f5dad134a31b43dd6</t>
-        </is>
-      </c>
-      <c r="CD25">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>DenseNet-121</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>UTC</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>validation/CAM ablation</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>completed; not promoted</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Test stronger masking against shortcut learning with the same CE DenseNet pipeline.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Retain current production checkpoint; no arm improved the complete selection trade-off.</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>No labeled test evaluation in this run; external YOLO-crop shift remains unresolved.</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/report.md</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>not archived in report folder</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>timm_densenet121_linear_native_cam</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>ImageNet pretrained</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>384x384 direct resize after square pad</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>Complete square-padded knee ROI; no center crop</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>LAB CLAHE clipLimit 1.25; SquarePad; direct Resize 384; ImageNet normalization</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Natural orientation; horizontal flip p=0.50; rotation +/-5 degrees; brightness/contrast 0.08; RandomErasing baseline p=0.10</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>Deterministic square-pad/CLAHE/resize; no stochastic augmentation</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Natural left/right orientation; no deterministic mirroring</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Full inverse-frequency WeightedRandomSampler</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>3-stage: 5 warm-up + 15 coarse + 10 fine-tune</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>5 head warm-up; 15 coarse; 10 full fine-tune</t>
-        </is>
-      </c>
-      <c r="X26">
-        <v>30</v>
-      </c>
-      <c r="Y26">
-        <v>26</v>
-      </c>
-      <c r="Z26">
-        <v>48</v>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>4 / Tesla T4</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>Cross-Entropy (CE)</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>AdamW</t>
-        </is>
-      </c>
-      <c r="AE26" t="inlineStr">
-        <is>
-          <t>CosineAnnealingLR</t>
-        </is>
-      </c>
-      <c r="AF26" t="inlineStr">
-        <is>
-          <t>warm-up 3e-4; coarse backbone 3e-5/head 3e-4; fine-tune 1e-5</t>
-        </is>
-      </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>1e-4</t>
-        </is>
-      </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>CUDA AMP</t>
-        </is>
-      </c>
-      <c r="AI26" t="inlineStr">
-        <is>
-          <t>global norm 1.0</t>
-        </is>
-      </c>
-      <c r="AJ26" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="AK26">
-        <v>42</v>
-      </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>0.55 QWK + 0.30 macro F1 + 0.15 macro AP</t>
-        </is>
-      </c>
-      <c r="AM26" t="inlineStr">
-        <is>
-          <t>Positive predicted-grade native CAM from five 1x1 class maps</t>
-        </is>
-      </c>
-      <c r="AN26" t="inlineStr">
-        <is>
-          <t>12x12</t>
-        </is>
-      </c>
-      <c r="AO26" t="inlineStr">
-        <is>
-          <t>5,778 train / 826 validation; test not read</t>
-        </is>
-      </c>
-      <c r="AP26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AQ26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AR26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AT26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AU26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AW26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AX26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AY26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AZ26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BA26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BB26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BC26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BD26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BE26">
-        <v>0.8037057762855189</v>
-      </c>
-      <c r="BF26">
-        <v>0.6832540391938888</v>
-      </c>
-      <c r="BG26">
-        <v>0.49019607843137253</v>
-      </c>
-      <c r="BH26">
-        <v>0.7298324958134197</v>
-      </c>
-      <c r="BI26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BJ26">
-        <v>0.756489263087215</v>
-      </c>
-      <c r="BK26">
-        <v>26</v>
-      </c>
-      <c r="BL26">
-        <v>826</v>
-      </c>
-      <c r="BM26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BO26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BP26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BQ26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BR26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BS26" t="inlineStr">
-        <is>
-          <t>Anatomy-gate failure rate 2.6634%; see per-case CSV in run folder.</t>
-        </is>
-      </c>
-      <c r="BT26">
-        <v>0.026634382566585957</v>
-      </c>
-      <c r="BU26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BV26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BW26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BX26" t="inlineStr">
-        <is>
-          <t>{"arm": "baseline_random_erasing", "best_epoch": "26", "cam_failure_rate": "0.026634382566585957", "checkpoint": "/content/drive/MyDrive/Models/densenet121_checkpoints/2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth", "grade1_recall": "0.49019607843137253", "macro_ap": "0.7298324958134197", "macro_f1": "0.6832540391938888", "qwk": "0.8037057762855189", "selection_score": "0.756489263087215"}</t>
-        </is>
-      </c>
-      <c r="BY26" t="inlineStr">
-        <is>
-          <t>Baseline random erasing had the best Grade 1 recall and macro F1; aggressive single cutout had the best QWK/AP but was not a production replacement.</t>
-        </is>
-      </c>
-      <c r="BZ26" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-      <c r="CA26" t="inlineStr">
-        <is>
-          <t>manual_artifact_metadata</t>
-        </is>
-      </c>
-      <c r="CB26" t="inlineStr">
-        <is>
-          <t>2026-07-28_02-00-33_963495_UTC_cutout_ablation/baseline_random_erasing/best_model.pth</t>
-        </is>
-      </c>
-      <c r="CC26" t="inlineStr">
-        <is>
-          <t>0c26982e344a339c247d4fc7d3a65672cade9c912d9f7f51b7f1a3256c430b28</t>
-        </is>
-      </c>
-      <c r="CD26">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>training/evaluation report</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>completed; separate model report</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Evaluate a larger multi-scale DenseNet backbone with ordinal training and Grad-CAM.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Retain as a documented candidate; QWK did not beat the best DenseNet-121 runs and Grade 1 recall is weak.</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Report does not provide an exact UTC run timestamp or checkpoint provenance; do not use as an exact production record.</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>dense_net_201.ipynb (path not present in report folder)</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>checkpoints/densenet201</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Multi-scale DenseNet-201; pooled transition-2, transition-3, and norm5 features</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>ImageNet pretrained</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>300x300</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>Square-padded knee ROI; exact crop provenance not documented</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>Square padding; CLAHE; grayscale normalization; resize as configured</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Horizontal flip p=0.50; capped rotation; small RandomErasing; no color jitter</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>Deterministic preprocessing; exact sequence not fully recorded</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Natural/symmetric laterality; exact policy not recorded</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Balanced WeightedRandomSampler in warm-up/coarse stages; stage-3 natural skew</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>3-stage warm-up + coarse + fine-tune</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>5 head warm-up; 25 coarse; 15 focal-CORN fine-tune (per configuration guide)</t>
-        </is>
-      </c>
-      <c r="X27">
-        <v>45</v>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr">
-        <is>
-          <t>CORN; Focal CORN in final stage</t>
-        </is>
-      </c>
-      <c r="AC27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>AdamW</t>
-        </is>
-      </c>
-      <c r="AE27" t="inlineStr">
-        <is>
-          <t>Cosine annealing; eta_min 1e-7</t>
-        </is>
-      </c>
-      <c r="AF27" t="inlineStr">
-        <is>
-          <t>backbone 1e-5; head 1e-4; final 1e-5</t>
-        </is>
-      </c>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>1e-4 stages 1/2; 1e-3 stage 3</t>
-        </is>
-      </c>
-      <c r="AH27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AI27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AJ27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AK27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AL27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AM27" t="inlineStr">
-        <is>
-          <t>Grad-CAM over norm5</t>
-        </is>
-      </c>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="AO27" t="inlineStr">
-        <is>
-          <t>1,656-image test split; patient grouping not documented</t>
-        </is>
-      </c>
-      <c r="AP27">
-        <v>1656</v>
-      </c>
-      <c r="AQ27">
-        <v>0.6624</v>
-      </c>
-      <c r="AR27">
-        <v>0.7763</v>
-      </c>
-      <c r="AS27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AT27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AU27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV27">
-        <v>0.63</v>
-      </c>
-      <c r="AW27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AX27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AY27">
-        <v>0.6948</v>
-      </c>
-      <c r="AZ27">
-        <v>0.8812</v>
-      </c>
-      <c r="BA27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BB27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BC27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BD27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BE27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BF27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BG27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BH27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BI27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BJ27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BK27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BL27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BM27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BO27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BP27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BQ27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BR27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BS27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BT27" t="inlineStr">
-        <is>
-          <t>288 / 826</t>
-        </is>
-      </c>
-      <c r="BU27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BV27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BW27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BX27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BY27" t="inlineStr">
-        <is>
-          <t>DenseNet-201 report recommends balanced stage-3 training and threshold review, but those recommendations were not validated in the documented run.</t>
-        </is>
-      </c>
-      <c r="BZ27" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-      <c r="CA27" t="inlineStr">
-        <is>
-          <t>report_markdown</t>
-        </is>
-      </c>
-      <c r="CB27" t="inlineStr">
-        <is>
-          <t>checkpoints/densenet201/best_model.pth</t>
-        </is>
-      </c>
-      <c r="CC27" t="inlineStr">
-        <is>
           <t>a8107b9cc7cc9242385f1facfcfc69c251f88697ed2df4dae8a43c1d66729b76</t>
         </is>
       </c>
-      <c r="CD27" t="inlineStr">
+      <c r="CD25" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -31600,12 +30278,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -31615,15 +30293,15 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>qwk</t>
+          <t>accuracy</t>
         </is>
       </c>
       <c r="F227">
-        <v>0.8126277960220584</v>
+        <v>0.6186</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31635,12 +30313,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -31650,15 +30328,15 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>macro_f1</t>
+          <t>qwk</t>
         </is>
       </c>
       <c r="F228">
-        <v>0.6819234872143023</v>
+        <v>0.7650</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31670,12 +30348,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -31685,15 +30363,15 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>grade1_recall</t>
+          <t>macro_f1</t>
         </is>
       </c>
       <c r="F229">
-        <v>0.45751633986928103</v>
+        <v>0.6451</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31705,12 +30383,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -31724,11 +30402,11 @@
         </is>
       </c>
       <c r="F230">
-        <v>0.7430301895958674</v>
+        <v>0.6756</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31740,12 +30418,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_double_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -31759,11 +30437,11 @@
         </is>
       </c>
       <c r="F231">
-        <v>0.762976862415803</v>
+        <v>0.7156</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31775,30 +30453,30 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>cam</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>qwk</t>
+          <t>joint_energy</t>
         </is>
       </c>
       <c r="F232">
-        <v>0.8202226229712083</v>
+        <v>0.8505</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31810,30 +30488,30 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>cam</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>macro_f1</t>
+          <t>border_energy</t>
         </is>
       </c>
       <c r="F233">
-        <v>0.68151148175952</v>
+        <v>0.0844</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
@@ -31845,448 +30523,203 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>2026-07-30 15:45:03.830205</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Production YOLO ROI robustness fine-tune</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>cam</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>grade1_recall</t>
+          <t>peak_inside_rate</t>
         </is>
       </c>
       <c r="F234">
-        <v>0.43137254901960786</v>
+        <v>1.0000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>notebook inline outputs</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>average_precision</t>
+          <t>accuracy</t>
         </is>
       </c>
       <c r="F235">
-        <v>0.7438495789896049</v>
+        <v>0.6624</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Cutout ablation: aggressive_single_cutout</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>selection_score</t>
+          <t>qwk</t>
         </is>
       </c>
       <c r="F236">
-        <v>0.7671533240104613</v>
+        <v>0.7763</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>qwk</t>
+          <t>macro_f1</t>
         </is>
       </c>
       <c r="F237">
-        <v>0.8037057762855189</v>
+        <v>0.63</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>macro_f1</t>
+          <t>average_precision</t>
         </is>
       </c>
       <c r="F238">
-        <v>0.6832540391938888</v>
+        <v>0.6948</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>repository artifact</t>
+          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>DenseNet-201</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-28 02:00:33.963495</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
+          <t>Optimized multi-scale DenseNet-201</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>grade1_recall</t>
+          <t>roc_auc</t>
         </is>
       </c>
       <c r="F239">
-        <v>0.49019607843137253</v>
+        <v>0.8812</v>
       </c>
       <c r="G239" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>DenseNet-121</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr">
-        <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
-        </is>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>average_precision</t>
-        </is>
-      </c>
-      <c r="F240">
-        <v>0.7298324958134197</v>
-      </c>
-      <c r="G240" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>DenseNet-121</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>2026-07-28 02:00:33.963495</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>Cutout ablation: baseline_random_erasing</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>validation</t>
-        </is>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>selection_score</t>
-        </is>
-      </c>
-      <c r="F241">
-        <v>0.756489263087215</v>
-      </c>
-      <c r="G241" t="inlineStr">
-        <is>
-          <t>repository artifact</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>accuracy</t>
-        </is>
-      </c>
-      <c r="F242">
-        <v>0.6624</v>
-      </c>
-      <c r="G242" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>qwk</t>
-        </is>
-      </c>
-      <c r="F243">
-        <v>0.7763</v>
-      </c>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="D244" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>macro_f1</t>
-        </is>
-      </c>
-      <c r="F244">
-        <v>0.63</v>
-      </c>
-      <c r="G244" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>average_precision</t>
-        </is>
-      </c>
-      <c r="F245">
-        <v>0.6948</v>
-      </c>
-      <c r="G245" t="inlineStr">
-        <is>
-          <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>DenseNet-201</t>
-        </is>
-      </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>Optimized multi-scale DenseNet-201</t>
-        </is>
-      </c>
-      <c r="D246" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>roc_auc</t>
-        </is>
-      </c>
-      <c r="F246">
-        <v>0.8812</v>
-      </c>
-      <c r="G246" t="inlineStr">
         <is>
           <t>docs/report/dense_net_201/dense_net_201_test_results.md</t>
         </is>

</xml_diff>